<commit_message>
Add quote-banner block for chairman masthead
The From Our Chairman masthead was migrated as columns-feature (small image +
text), but the source is a distinct design: a full-bleed portrait with an
overlapping translucent mint quote card (decorative quote marks, centered quote,
attribution). Added a dedicated quote-banner block + parser and wired it into
the letter-page import in place of columns-feature.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-letter-page.report.xlsx
+++ b/tools/importer/reports/import-letter-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="58">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,22 +37,43 @@
     <t>url</t>
   </si>
   <si>
+    <t>community-stewardship.report.json</t>
+  </si>
+  <si>
+    <t>["chapter-nav","callout-case-study"]</t>
+  </si>
+  <si>
+    <t>community-stewardship</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>chapter-page</t>
+  </si>
+  <si>
+    <t>2026-07-09T07:24:34.299Z</t>
+  </si>
+  <si>
+    <t>Community Stewardship | Temasek Review 2026</t>
+  </si>
+  <si>
+    <t>https://www.temasekreview.com.sg/community-stewardship.html</t>
+  </si>
+  <si>
     <t>from-our-chairman.report.json</t>
   </si>
   <si>
-    <t>["columns-feature"]</t>
+    <t>["quote-banner"]</t>
   </si>
   <si>
     <t>from-our-chairman</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>letter-page</t>
   </si>
   <si>
-    <t>2026-07-08T17:59:27.046Z</t>
+    <t>2026-07-09T08:43:42.170Z</t>
   </si>
   <si>
     <t>From Our Chairman | Temasek Review 2026</t>
@@ -82,25 +103,88 @@
     <t>https://www.temasekreview.com.sg/</t>
   </si>
   <si>
+    <t>institution.report.json</t>
+  </si>
+  <si>
+    <t>["chapter-nav"]</t>
+  </si>
+  <si>
+    <t>institution</t>
+  </si>
+  <si>
+    <t>2026-07-09T07:01:49.499Z</t>
+  </si>
+  <si>
+    <t>Institution | Temasek Review 2026</t>
+  </si>
+  <si>
+    <t>https://www.temasekreview.com.sg/institution.html</t>
+  </si>
+  <si>
+    <t>media-centre.report.json</t>
+  </si>
+  <si>
+    <t>media-centre</t>
+  </si>
+  <si>
+    <t>2026-07-09T07:26:15.558Z</t>
+  </si>
+  <si>
+    <t>Media Centre | Temasek Review 2026</t>
+  </si>
+  <si>
+    <t>https://www.temasekreview.com.sg/media-centre.html</t>
+  </si>
+  <si>
+    <t>performance-and-portfolio.report.json</t>
+  </si>
+  <si>
+    <t>["chapter-nav","callout-case-study","callout-case-study","callout-case-study","callout-case-study","logo-grid","logo-grid","logo-grid","logo-grid","logo-grid"]</t>
+  </si>
+  <si>
+    <t>performance-and-portfolio</t>
+  </si>
+  <si>
+    <t>2026-07-09T06:46:13.569Z</t>
+  </si>
+  <si>
+    <t>Performance &amp; Portfolio | Temasek Review 2026</t>
+  </si>
+  <si>
+    <t>https://www.temasekreview.com.sg/performance-and-portfolio.html</t>
+  </si>
+  <si>
     <t>strategy.report.json</t>
   </si>
   <si>
-    <t>["callout-case-study","callout-case-study","callout-case-study","callout-case-study","logo-grid","logo-grid","logo-grid"]</t>
+    <t>["chapter-nav","callout-case-study","callout-case-study","callout-case-study","callout-case-study","logo-grid","logo-grid","logo-grid"]</t>
   </si>
   <si>
     <t>strategy</t>
   </si>
   <si>
-    <t>chapter-page</t>
-  </si>
-  <si>
-    <t>2026-07-08T17:18:27.256Z</t>
+    <t>2026-07-09T05:11:06.201Z</t>
   </si>
   <si>
     <t>Strategy | Temasek Review 2026</t>
   </si>
   <si>
     <t>https://www.temasekreview.com.sg/strategy.html</t>
+  </si>
+  <si>
+    <t>sustainability.report.json</t>
+  </si>
+  <si>
+    <t>sustainability</t>
+  </si>
+  <si>
+    <t>2026-07-09T07:10:36.183Z</t>
+  </si>
+  <si>
+    <t>Sustainability | Temasek Review 2026</t>
+  </si>
+  <si>
+    <t>https://www.temasekreview.com.sg/sustainability.html</t>
   </si>
 </sst>
 </file>
@@ -489,12 +573,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="31" customWidth="1"/>
+    <col min="1" max="1" width="39" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="19" customWidth="1"/>
+    <col min="3" max="3" width="27" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="49" customWidth="1"/>
@@ -605,6 +689,136 @@
         <v>29</v>
       </c>
     </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>55</v>
+      </c>
+      <c r="G9" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" t="s">
+        <v>57</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add chapter-nav to letter-page (chairman) import
The chairman page's .contenttopnav was leaking in as raw prose links above the
masthead because the letter-page import had no chapter-nav mapping. Add the
chapter-nav block (hierarchy-driven prev/current/next) so it renders as the
styled nav bar like the chapter pages, instead of plain paragraphs.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-letter-page.report.xlsx
+++ b/tools/importer/reports/import-letter-page.report.xlsx
@@ -64,7 +64,7 @@
     <t>from-our-chairman.report.json</t>
   </si>
   <si>
-    <t>["quote-banner"]</t>
+    <t>["chapter-nav","quote-banner"]</t>
   </si>
   <si>
     <t>from-our-chairman</t>
@@ -73,7 +73,7 @@
     <t>letter-page</t>
   </si>
   <si>
-    <t>2026-07-09T08:43:42.170Z</t>
+    <t>2026-07-09T08:50:30.799Z</t>
   </si>
   <si>
     <t>From Our Chairman | Temasek Review 2026</t>

</xml_diff>